<commit_message>
Added baffle length w/ liner
I discovered for Baffle Box Calc : Calculation 1, it's possible for the baffle length to be smaller than the AirGap. Having a smaller baffle than the AirGap is not good as this would cause a straight path down the center for sound and air to travel through defeating the purpose of the baffles. I added a new cell 'w/ liner' that adds the liner thickness to the baffle length. This measurement is then compared against the AirGap to determine if meets standards.
</commit_message>
<xml_diff>
--- a/Calculations.xlsx
+++ b/Calculations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sekthree\Documents\hometheater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9953E1EF-6025-4CE0-ABD4-6214461EE53A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D971C924-AA0C-4E9E-BFC4-D70D0BA60435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DB8C7B79-F667-4C5F-9663-F5C375358015}"/>
   </bookViews>
@@ -54,6 +54,7 @@
     <author>tc={B4934FCD-3175-4E8B-82F8-C8E5289A5A80}</author>
     <author>tc={AADA5476-0F4E-4CAB-BB1D-11BC5BE6E828}</author>
     <author>tc={97BB840E-1454-43F8-9637-7433D8598001}</author>
+    <author>tc={4CF90B3C-2E93-4A0A-85D7-42B28CF9BCB5}</author>
   </authors>
   <commentList>
     <comment ref="O6" authorId="0" shapeId="0" xr:uid="{EEC4EF2A-D5BB-4496-80B1-218C6BE1D6C5}">
@@ -128,12 +129,21 @@
     Length of the wood from the internal wood wall. 1” Liner should be added to the end. </t>
       </text>
     </comment>
+    <comment ref="I13" authorId="9" shapeId="0" xr:uid="{4CF90B3C-2E93-4A0A-85D7-42B28CF9BCB5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Adjust either Air Velocity (FPM) or Ext. Width/Height till this is Green.
+This means the baffle with liner are GREATER than the air gap preventing line of sight path.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -155,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="118">
   <si>
     <t>Ceiling Variables</t>
   </si>
@@ -496,23 +506,26 @@
   </si>
   <si>
     <t>B4. Create Your Box. Take Width and Height from ductulator.com and plug into values below. Enter baffle count. Or just start entering values, CalcFPM will tell you if good.</t>
+  </si>
+  <si>
+    <t>1. Enter Length and width of ceiling. Width can also be height of a wall however placement does not incorporate 3"-6" placement of top and bottom rows.</t>
+  </si>
+  <si>
+    <t>by</t>
+  </si>
+  <si>
+    <t>sekthree</t>
+  </si>
+  <si>
+    <t>w/ liner</t>
   </si>
   <si>
     <t>First thing.. Like most of all DIY'ers, I AM NOT AN EXPERT. These calculations are NOT absoluate. This is all empirical data.
 Description: Calculate the baffle box size needed for a rooms requirements for HVAC vents. Standard requirements for a home residents is that the air in a room should be exchanged 6 times per hour. By providing a rooms dimensions (LxWxH) the Cubit Fee per Minute (CFM) that is needed is calculated for this exchange to take place. For every occupant of a room it's also recommended for 15 CFM to occur, for six people that's 90 CFM, so unless crowded in a closet most Loads should suffice.
 When air is supplied a rushing/wooshing sound and sometimes a whistle can be audible by the fast moving air. This is due to the speed of the air being supplied within a given boxed area. To alleviate this issue the air velocity can be lowered and surfaces can be affixed with sound absorbing material. The recommended velocity for air to be supplied so as to not be audible is roughly 300 Feet Per Minute (FPM). By providing this value the box is calculated to meet this requirement, however this is not a static value and can be changed if desired. Think of water moving through and releasing from a pipe: when minimum slow moving water there's no noise (other than the drip hitting a surface), but when tons of water is rushing through a small pipe it makes a garbbablebblebele sound, lik a firehose, shower, or faucet.
 When calculating a box, it's assumed to be using 3/4" plywood and 1" ductboard. These values are not static and can be updated. Two types of boxes are calculated. 
-The 1st is calculated based on size restrictions provided, but only two values: Width and Height, This is because the third value (Length) is what is calculated in order to meet CFM &amp; FPM requirements. Recommended for instances of placing baffle boxes between ceiling joists or in soffits. The amount of baffles can also be given which will affect the box size. Each baffle provides reduction in decibels, however I've read diminishing returns occurs beyond three baffles. The golden ratio is also used to calculate baffle placement. Staggered baffles help disrupt air and sound to reduce static pressure and standing waves. Baffle placement is provided in the Absoluate On Center Position column. This is to be measured from the entrance side on the inside of the box against the wood not the liner. The measurement marks the CENTER of the wood baffle. Baffles should be placed along the wider part (width or height) of the box, the calculations try to take this into considerations. Ex. if you have a box 20"x13", the baffle will be cut and placed against the 20" side giving an ~11" baffle (wood)  with ~4" gap (between liners). Lastely included is to calculate from the "Load CFM" or from "CFM minus soffit" area. If soffits are in the room this technically takes away from a rooms cubic area and thus from it's CFM. It's recommended to use the Load CFM as occupancy and heat from equipment factor into room comfort, but in the event you're working with a small area for baffle placement and want to squeeze out as much as you can, removing soffit area can be done. Soffits assume to be identical.
+The 1st is calculated based on size restrictions provided, but only two values: Width and Height, This is because the third value (Length) is what is calculated in order to meet CFM &amp; FPM requirements. Recommended for instances of placing baffle boxes between ceiling joists or in soffits. The amount of baffles can also be given which will affect the box size. Each baffle provides reduction in decibels, however I've read diminishing returns occurs beyond three baffles. The golden ratio is also used to calculate baffle placement. Staggered baffles help disrupt air and sound to reduce static pressure and standing waves. Baffle placement is provided in the Absoluate On Center Position column. This is to be measured from the entrance side on the inside of the box against the wood not the liner. The measurement marks the CENTER of the wood baffle. Baffles should be placed along the wider part (width or height) of the box, the calculations try to take this into considerations. Ex. if you have a box 20"x13", the baffle will be cut and placed against the 20" side giving an ~11" baffle (wood)  with ~4" gap (between liners). Lastely included is to calculate from the "Load CFM" or from "CFM minus soffit" area. If soffits are in the room this technically takes away from a rooms cubic area and thus from it's CFM. It's recommended to use the Load CFM as occupancy and heat from equipment factor into room comfort, but in the event you're working with a small area for baffle placement and want to squeeze out as much as you can, removing soffit area can be done. Soffits assume to be identical. I've added a baffle length w/ liner. This measurement MUST be larger than the gap otherwise a straight path down the center will occur for sound and air to travel through. Increase FPM or external width or height measurements until baffle length w/ liner is GREEN.
 The 2nd is calculated based on internal duct size being equal throughout the box with no external measurement restrictions. This is used for instances when placing the baffle box outside of the room like in an adjacent room. The website provided should provide the exact measurements for internal duct area to meet the CFM &amp; FPM requirements. These variables are then transferred to this sheet to provide the box size needed to match the internal duct size. Although the sheet also validates measurements by calculating the FPM from the internal duct size provided; green - good, red - bad. Duct sizes can be entered without visiting the website, and the sheet will show if requirements are met or not. Baffle count can also be entered, see above for baffle count explaination.</t>
-  </si>
-  <si>
-    <t>1. Enter Length and width of ceiling. Width can also be height of a wall however placement does not incorporate 3"-6" placement of top and bottom rows.</t>
-  </si>
-  <si>
-    <t>by</t>
-  </si>
-  <si>
-    <t>sekthree</t>
   </si>
 </sst>
 </file>
@@ -671,7 +684,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -696,6 +709,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="13" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -714,28 +741,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="13" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill>
@@ -754,6 +766,27 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -881,7 +914,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{99876655-E06A-4C27-B677-5F7A21019C72}" name="Table1" displayName="Table1" ref="A3:C7" totalsRowShown="0" headerRowDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{99876655-E06A-4C27-B677-5F7A21019C72}" name="Table1" displayName="Table1" ref="A3:C7" totalsRowShown="0" headerRowDxfId="12">
   <autoFilter ref="A3:C7" xr:uid="{99876655-E06A-4C27-B677-5F7A21019C72}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{2074FFFD-46EA-49A3-84F3-1445992B9E0E}" name="Ceiling Variables"/>
@@ -895,7 +928,7 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BBAB1DFE-2A65-4E6C-BEA6-2E323EBACC11}" name="Table5" displayName="Table5" ref="A10:C16" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{8AB85CC7-9D5F-4E9D-82CF-D83CE313A743}" name="Column1" headerRowDxfId="8" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{8AB85CC7-9D5F-4E9D-82CF-D83CE313A743}" name="Column1" headerRowDxfId="11" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{C5A989E4-834D-422D-AD53-E59E3D1107F7}" name="Column2"/>
     <tableColumn id="3" xr3:uid="{CB0D3CF6-A70F-47AC-9B1F-15C0BD8AAA8D}" name="Column3"/>
   </tableColumns>
@@ -906,7 +939,7 @@
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C5159225-FBEB-498D-AA96-6C40AA0CBBAC}" name="Table6" displayName="Table6" ref="A19:C25" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0E11655C-CED4-417B-A346-742C93C65A00}" name="Column1" headerRowDxfId="6" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{0E11655C-CED4-417B-A346-742C93C65A00}" name="Column1" headerRowDxfId="9" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{7A083905-B44C-4636-8050-67665F3B762C}" name="Column2"/>
     <tableColumn id="3" xr3:uid="{8DE6389C-5722-4EFB-886C-36C50B464F3E}" name="Column3"/>
   </tableColumns>
@@ -1269,6 +1302,10 @@
   <threadedComment ref="H12" dT="2026-03-23T03:04:38.26" personId="{80B567F5-4A80-4E80-92D4-94B755173946}" id="{97BB840E-1454-43F8-9637-7433D8598001}">
     <text xml:space="preserve">Length of the wood from the internal wood wall. 1” Liner should be added to the end. </text>
   </threadedComment>
+  <threadedComment ref="I13" dT="2026-03-30T19:15:23.69" personId="{80B567F5-4A80-4E80-92D4-94B755173946}" id="{4CF90B3C-2E93-4A0A-85D7-42B28CF9BCB5}">
+    <text>Adjust either Air Velocity (FPM) or Ext. Width/Height till this is Green.
+This means the baffle with liner are GREATER than the air gap preventing line of sight path.</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -1287,25 +1324,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
     </row>
     <row r="2" spans="1:17" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6"/>
@@ -1324,10 +1361,10 @@
       <c r="N2" s="6"/>
       <c r="O2" s="6"/>
       <c r="P2" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q2" s="6" t="s">
         <v>115</v>
-      </c>
-      <c r="Q2" s="6" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -1352,7 +1389,7 @@
         <v>5</v>
       </c>
       <c r="E4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
@@ -1687,66 +1724,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
     </row>
     <row r="2" spans="1:16" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="30"/>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30" t="s">
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="P2" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="P2" s="30" t="s">
-        <v>116</v>
-      </c>
     </row>
     <row r="3" spans="1:16" ht="335.4" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
+      <c r="A3" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
@@ -1841,7 +1878,7 @@
       <c r="B7" s="4">
         <v>237</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="16" t="s">
         <v>11</v>
       </c>
       <c r="D7" t="s">
@@ -1878,11 +1915,11 @@
       </c>
       <c r="O7">
         <f>L9</f>
-        <v>7.4968864864864866</v>
+        <v>6.8607382239382249</v>
       </c>
       <c r="P7">
         <f>O7</f>
-        <v>7.4968864864864866</v>
+        <v>6.8607382239382249</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
@@ -1890,9 +1927,9 @@
         <v>42</v>
       </c>
       <c r="B8" s="4">
-        <v>133</v>
-      </c>
-      <c r="C8" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" s="16" t="s">
         <v>11</v>
       </c>
       <c r="D8" t="s">
@@ -1909,7 +1946,7 @@
         <v>61</v>
       </c>
       <c r="I8" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" t="s">
         <v>17</v>
@@ -1929,11 +1966,11 @@
       </c>
       <c r="O8">
         <f>O7</f>
-        <v>7.4968864864864866</v>
+        <v>6.8607382239382249</v>
       </c>
       <c r="P8">
         <f>SUM(1,P7,1,(B17/2))</f>
-        <v>9.8562614864864866</v>
+        <v>9.220113223938224</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
@@ -1967,7 +2004,7 @@
       </c>
       <c r="L9">
         <f>I10*1.1</f>
-        <v>7.4968864864864866</v>
+        <v>6.8607382239382249</v>
       </c>
       <c r="M9" t="s">
         <v>11</v>
@@ -1977,11 +2014,11 @@
       </c>
       <c r="O9">
         <f>O7*POWER(I9,2)</f>
-        <v>19.626279058248652</v>
+        <v>17.960891254165254</v>
       </c>
       <c r="P9">
         <f>SUM(B17,1,P8,O9,1)</f>
-        <v>32.201290544735137</v>
+        <v>29.899754478103478</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
@@ -1990,7 +2027,7 @@
       </c>
       <c r="B10">
         <f>PRODUCT(feetCheck(C7,B7),feetCheck(C8,B8))</f>
-        <v>218.89583333333334</v>
+        <v>233.70833333333334</v>
       </c>
       <c r="C10" t="s">
         <v>77</v>
@@ -2010,7 +2047,7 @@
       </c>
       <c r="I10">
         <f>(IF(O5="CFM Minus Soffit",E14,B14)*144)/(B15*IF(L6&gt;=L7,L6,L7))</f>
-        <v>6.8153513513513513</v>
+        <v>6.2370347490347493</v>
       </c>
       <c r="J10" t="s">
         <v>11</v>
@@ -2020,7 +2057,7 @@
       </c>
       <c r="L10">
         <f>(IF(O5="CFM Minus Soffit",E14,B14)*144)/L8</f>
-        <v>213.81494435612083</v>
+        <v>228.28362480127186</v>
       </c>
       <c r="M10" t="s">
         <v>68</v>
@@ -2030,11 +2067,11 @@
       </c>
       <c r="O10">
         <f>IF(I8&gt;=N10,O7*I9,0)</f>
-        <v>0</v>
+        <v>11.100674446332048</v>
       </c>
       <c r="P10">
         <f>IF(I8&gt;=N10,SUM(B17,1,P9,O10,1),0)</f>
-        <v>0</v>
+        <v>43.719178924435525</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
@@ -2043,7 +2080,7 @@
       </c>
       <c r="B11">
         <f>PRODUCT(feetCheck(C7,B7),feetCheck(C8,B8),feetCheck(C9,B9))</f>
-        <v>1641.71875</v>
+        <v>1752.8125</v>
       </c>
       <c r="C11" t="s">
         <v>58</v>
@@ -2064,7 +2101,7 @@
       </c>
       <c r="I11">
         <f ca="1">SUM(OFFSET(O7,0,0,I8+1,1))+(I8*SUM(B18,B17,B18))+SUM(B17,B18,B18,B17)</f>
-        <v>43.495052031221626</v>
+        <v>54.376792148373752</v>
       </c>
       <c r="J11" t="s">
         <v>11</v>
@@ -2074,7 +2111,7 @@
       </c>
       <c r="L11">
         <f>(IF(O5="CFM Minus Soffit",E14,B14)*144)/(IF(L6&gt;=L7,L6,L7)*I10)</f>
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="M11" t="s">
         <v>68</v>
@@ -2114,7 +2151,7 @@
       </c>
       <c r="I12">
         <f>IF(L6&gt;=L7,L6,L7)-I10</f>
-        <v>4.7471486486486487</v>
+        <v>5.3254652509652507</v>
       </c>
       <c r="J12" t="s">
         <v>11</v>
@@ -2126,9 +2163,19 @@
       </c>
       <c r="B13">
         <f>B11/60*B12</f>
-        <v>9.5766927083333329</v>
+        <v>10.224739583333333</v>
       </c>
       <c r="G13" s="6"/>
+      <c r="H13" t="s">
+        <v>116</v>
+      </c>
+      <c r="I13">
+        <f>I12+B18</f>
+        <v>6.3254652509652507</v>
+      </c>
+      <c r="J13" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -2136,7 +2183,7 @@
       </c>
       <c r="B14" s="10">
         <f>B11/10</f>
-        <v>164.171875</v>
+        <v>175.28125</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
@@ -2146,7 +2193,7 @@
       </c>
       <c r="E14">
         <f>SUM(B11,-E12)/10</f>
-        <v>154.18715277777778</v>
+        <v>165.29652777777778</v>
       </c>
       <c r="F14" t="s">
         <v>45</v>
@@ -2167,7 +2214,7 @@
         <v>69</v>
       </c>
       <c r="B15" s="4">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="C15" t="s">
         <v>68</v>
@@ -2176,16 +2223,16 @@
     </row>
     <row r="16" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G16" s="6"/>
-      <c r="H16" s="17" t="s">
+      <c r="H16" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
     </row>
     <row r="17" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
@@ -2197,15 +2244,15 @@
       <c r="C17" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="27"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
     </row>
     <row r="18" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
@@ -2220,33 +2267,33 @@
       <c r="G18" s="6"/>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
-      <c r="J18" s="18" t="s">
+      <c r="J18" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
       <c r="N18" s="11"/>
       <c r="O18" s="11"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="G19" s="6"/>
-      <c r="H19" s="17" t="s">
+      <c r="H19" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="25"/>
+      <c r="M19" s="25"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="25"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="B20" s="19"/>
+      <c r="B20" s="27"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
@@ -2263,14 +2310,14 @@
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="28"/>
       <c r="G21" s="6"/>
       <c r="H21" s="4" t="s">
         <v>55</v>
@@ -2283,12 +2330,12 @@
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="20"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
       <c r="G22" s="6"/>
       <c r="H22" s="4" t="s">
         <v>54</v>
@@ -2301,12 +2348,12 @@
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="20"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
       <c r="G23" s="6"/>
       <c r="H23" s="4" t="s">
         <v>53</v>
@@ -2319,12 +2366,12 @@
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="20"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
       <c r="G24" s="6"/>
       <c r="H24" t="s">
         <v>52</v>
@@ -2335,35 +2382,35 @@
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A25" s="20"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
       <c r="G25" s="6"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
       <c r="G26" s="6"/>
       <c r="H26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
       <c r="G27" s="6"/>
       <c r="H27" t="s">
         <v>50</v>
@@ -2391,12 +2438,12 @@
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A28" s="16"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="6"/>
       <c r="H28" t="s">
         <v>4</v>
@@ -2424,12 +2471,12 @@
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="A29" s="24"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
       <c r="G29" s="6"/>
       <c r="H29" t="s">
         <v>10</v>
@@ -2469,7 +2516,7 @@
       </c>
       <c r="M30">
         <f>(B14*144)/M29</f>
-        <v>295.50937499999998</v>
+        <v>315.50625000000002</v>
       </c>
       <c r="N30" t="s">
         <v>68</v>
@@ -2509,25 +2556,36 @@
     <mergeCell ref="A21:F25"/>
   </mergeCells>
   <conditionalFormatting sqref="B14">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>$O$5="Load CFM"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>$O$5="CFM Minus Soffit"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I13">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>$I$13=$I$10</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>$I$13&gt;$I$10</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>$I$13&lt;$I$10</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L10:M10 M11">
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="2" priority="8">
       <formula>$L$10&gt;$B$15</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M30">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>$M$30&gt;$B$15</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>$M$30&lt;=$B$15</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2569,22 +2627,22 @@
   </cols>
   <sheetData>
     <row r="5" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
     </row>
     <row r="6" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21" t="s">
+      <c r="D6" s="29"/>
+      <c r="E6" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="21"/>
+      <c r="F6" s="29"/>
     </row>
     <row r="7" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
@@ -2601,17 +2659,17 @@
       </c>
     </row>
     <row r="8" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C8" s="26">
-        <v>7.4968864860000002</v>
-      </c>
-      <c r="D8" s="23" t="s">
+      <c r="C8" s="19">
+        <v>142</v>
+      </c>
+      <c r="D8" s="17" t="s">
         <v>11</v>
       </c>
       <c r="E8" cm="1">
         <f t="array" ref="E8">_xlfn.IFS(F8="inches",inchesCheck(D8,C8),F8="feet",feetCheck(D8,C8))</f>
-        <v>0.62474054050000005</v>
-      </c>
-      <c r="F8" s="23" t="s">
+        <v>11.833333333333334</v>
+      </c>
+      <c r="F8" s="17" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2621,16 +2679,16 @@
       </c>
     </row>
     <row r="10" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="E10" s="24" cm="1">
+      <c r="E10" s="18" cm="1">
         <f t="array" ref="E10">MROUND(inchesCheck(D8,$C$8),0.03125)</f>
-        <v>7.5</v>
+        <v>142</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="E11" s="25" t="s">
+      <c r="E11" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2640,9 +2698,9 @@
       </c>
     </row>
     <row r="13" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="E13" s="25" cm="1">
+      <c r="E13" cm="1">
         <f t="array" ref="E13">FLOOR(feetCheck($D$8,TRUNC($C$8)),1)</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F13" t="s">
         <v>106</v>
@@ -2651,7 +2709,7 @@
     <row r="14" spans="3:6" x14ac:dyDescent="0.3">
       <c r="E14" s="2" cm="1">
         <f t="array" ref="E14">IF(D8="feet",inchesCheck($D$8,$C$8-TRUNC($C$8)),MOD(C8,12))</f>
-        <v>7.4968864860000002</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
         <v>11</v>

</xml_diff>